<commit_message>
Add BB.mq5 result to comparison report
2024-2026 validated run: PF 1.27, net +3546.33 on $10k, 3068 trades,
67.5% win rate. Drawdown notably higher than other bots (16.5%
balance / 22.4% equity vs prior max 5.8%) -- flagged in notes;
confirmed structural (correlated multi-TF entries) via permutation
test, not a fragile-edge symptom.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/XAUUSD_Bot_Comparison.xlsx
+++ b/reports/XAUUSD_Bot_Comparison.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="30" customWidth="1" style="21" min="1" max="1"/>
@@ -580,6 +580,11 @@
           <t>EMA/BB Cross (M5)</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>BB (6TF, EMA-chase)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -605,6 +610,9 @@
       <c r="G5" s="14" t="n">
         <v>1175</v>
       </c>
+      <c r="H5" s="14" t="n">
+        <v>3546.33</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -630,6 +638,9 @@
       <c r="G6" s="15" t="n">
         <v>1.2215</v>
       </c>
+      <c r="H6" s="15" t="n">
+        <v>1.27</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -655,6 +666,9 @@
       <c r="G7" s="16" t="n">
         <v>1781</v>
       </c>
+      <c r="H7" s="16" t="n">
+        <v>3068</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -680,6 +694,9 @@
       <c r="G8" s="17" t="n">
         <v>0.4043</v>
       </c>
+      <c r="H8" s="17" t="n">
+        <v>0.675</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -711,6 +728,10 @@
         <f>1-G8</f>
         <v/>
       </c>
+      <c r="H9" s="17">
+        <f>1-H8</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -736,6 +757,9 @@
       <c r="G10" s="14" t="n">
         <v>9</v>
       </c>
+      <c r="H10" s="14" t="n">
+        <v>8.08</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -761,6 +785,9 @@
       <c r="G11" s="14" t="n">
         <v>-5</v>
       </c>
+      <c r="H11" s="14" t="n">
+        <v>-13.24</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -792,6 +819,10 @@
         <f>G8*G10+G9*G11</f>
         <v/>
       </c>
+      <c r="H12" s="18">
+        <f>H8*H10+H9*H11</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -817,6 +848,9 @@
       <c r="G13" s="14" t="n">
         <v>132</v>
       </c>
+      <c r="H13" s="14" t="n">
+        <v>1857.52</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -842,6 +876,9 @@
       <c r="G14" s="19" t="n">
         <v>0.0118</v>
       </c>
+      <c r="H14" s="19" t="n">
+        <v>0.1649</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -867,6 +904,9 @@
       <c r="G15" s="14" t="n">
         <v>132</v>
       </c>
+      <c r="H15" s="14" t="n">
+        <v>2523.99</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -892,6 +932,9 @@
       <c r="G16" s="19" t="n">
         <v>0.0118</v>
       </c>
+      <c r="H16" s="19" t="n">
+        <v>0.224</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -917,6 +960,9 @@
       <c r="G17" s="16" t="n">
         <v>982</v>
       </c>
+      <c r="H17" s="16" t="n">
+        <v>984</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -948,6 +994,10 @@
         <f>G5/G17</f>
         <v/>
       </c>
+      <c r="H18" s="18">
+        <f>H5/H17</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -979,6 +1029,10 @@
         <f>G7/G17</f>
         <v/>
       </c>
+      <c r="H19" s="15">
+        <f>H7/H17</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="15.5" customHeight="1" s="21">
       <c r="A22" s="10" t="inlineStr">
@@ -1018,6 +1072,11 @@
           <t>EMA/BB Cross (M5)</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>BB (6TF, EMA-chase)</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="23" customHeight="1" s="21">
       <c r="A24" s="12" t="inlineStr">
@@ -1050,6 +1109,11 @@
           <t>EMA(20) crosses BB(20,2.0) mid -&gt; instant market buy/sell, SL 5 / TP 9 (real price distance, broker-independent)</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>BB(20,2.0) x6 TF: M1/M5/M15/M30/H1 (H4 orig off)</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="34.5" customHeight="1" s="21">
       <c r="A25" s="12" t="inlineStr">
@@ -1082,6 +1146,11 @@
           <t>Hour filter: blocks server hours 10, 18, 19</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>THS/THB: instant market, bid/ask vs band, TP=band, thr=4</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="34.5" customHeight="1" s="21">
       <c r="A26" s="12" t="inlineStr">
@@ -1114,6 +1183,11 @@
           <t>Minute-of-hour filter: buy only at :05/:40/:50, sell only at :40</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>THS2/THB2 addon: limit at bar wick, TP=band, cancel after 1 bar</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="34.5" customHeight="1" s="21">
       <c r="A27" s="12" t="inlineStr">
@@ -1146,6 +1220,11 @@
           <t>No trend/volatility/pre-cross filter (tested, none improved results)</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>TP re-pegs every bar (EMA frac=0.6 orig, 0.667 addon), no fixed SL</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="34.5" customHeight="1" s="21">
       <c r="A28" s="12" t="inlineStr">
@@ -1174,6 +1253,11 @@
           <t>Max concurrent M5 positions: unlimited (0)</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Addon requires wick AND close both clear threshold (filters noise)</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="34.5" customHeight="1" s="21">
       <c r="A29" s="12" t="inlineStr">
@@ -1200,6 +1284,11 @@
       <c r="G29" t="inlineStr">
         <is>
           <t>Fixed lot 0.01</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Per-TF isolate switches: H4 orig off, M1 addon off (both underperformed)</t>
         </is>
       </c>
     </row>
@@ -1241,6 +1330,8 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="23" t="inlineStr">
         <is>
@@ -1308,6 +1399,41 @@
       <c r="A43" s="20" t="inlineStr">
         <is>
           <t>- Permutation test (5000 shuffles of trade outcomes against the fixed hour/minute rule): actual PF=1.2215 exceeded every one of the 5000 random draws (p=0.00000, null median PF=0.980) -- confirms the FIXED rule isn't random noise, but does not by itself prove the rule-discovery process (searching many hour/minute combos) is free of overfitting; the walk-forward result above is what actually tests that.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>BB.mq5: no fixed TP/SL -- TP chases toward latest close each bar (EMA),</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>closing the unbounded-loss failure mode a static TP had on trends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Validated via 70/30 split + 3-window walk-forward + permutation test</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>(drawdown clusters on correlated multi-TF entries during shared moves,</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>confirmed structural via permutation, not a fragile-edge symptom).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add preBB.mq5: BB signal EA rewrite (addon removed, M5/M15/M30/H1, %-scaled threshold)
Rewrote BB.mq5 into preBB.mq5: dropped the THS2/THB2 limit-fade addon and
M1/H4 timeframes, replaced the entry rule with one symmetric band-breakout
signal, switched the threshold from a fixed $ value to % of band price
(the $ version was regime-dependent as gold's price level shifted 2021-2026).
Validated via real MT5 Strategy Tester over 2021-2026: permutation test,
70/30 split, real walk-forward, equity/balance drawdown, and a repaint
check on the entry signal's band-value read. Wired defaults: K=0.55%,
per-TF chase fractions 0.6/0.5/0.75/0.5. Added to the bot comparison report
as a new column (old BB.mq5 column kept for reference).

Known open risk, documented in the report: 83% of backtest profit comes
from one 4-month window (2026 Jan-Apr) -- not yet forward-tested live/demo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/XAUUSD_Bot_Comparison.xlsx
+++ b/reports/XAUUSD_Bot_Comparison.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="27580" windowHeight="17740" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot Comparison" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="181029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -19,7 +19,7 @@
     <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,32 +41,50 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="9"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
       <color rgb="FF555555"/>
-      <sz val="9"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color rgb="FF555555"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -114,49 +132,52 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -522,818 +543,913 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="30" customWidth="1" style="21" min="1" max="1"/>
-    <col width="28" customWidth="1" style="21" min="2" max="5"/>
-    <col width="16" customWidth="1" style="21" min="6" max="6"/>
+    <col width="33.1796875" customWidth="1" style="18" min="1" max="1"/>
+    <col width="28" customWidth="1" style="18" min="2" max="5"/>
+    <col width="16" customWidth="1" style="18" min="6" max="6"/>
+    <col width="26.7265625" customWidth="1" style="18" min="7" max="7"/>
+    <col width="22.81640625" customWidth="1" style="18" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="21">
-      <c r="A1" s="22" t="inlineStr">
+    <row r="1" ht="18" customHeight="1" s="18">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>XAUUSD Bot Portfolio - Backtest Comparison</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Backtest period: 2024.01.01 - 2026.09.09 (982 days) - Real MT5 Strategy Tester, fixed lot 0.01, Model=Open prices (Model=1)</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+    <row r="4" ht="28" customHeight="1" s="18">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>RegimeBot (H1)</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>H1 Ratchet</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>M30 Ratchet</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>M15 Scalper</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>M5 Scalper</t>
         </is>
       </c>
-      <c r="G4" s="13" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>EMA/BB Cross (M5)</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>BB (6TF, EMA-chase)</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>preBB v6 (%K, 4TF)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Total Net Profit ($)</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="7" t="n">
         <v>2744.24</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="7" t="n">
         <v>1689.42</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="7" t="n">
         <v>3015.39</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="7" t="n">
         <v>5035.78</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F5" s="7" t="n">
         <v>1647.24</v>
       </c>
-      <c r="G5" s="14" t="n">
+      <c r="G5" s="7" t="n">
         <v>1175</v>
       </c>
-      <c r="H5" s="14" t="n">
+      <c r="H5" s="7" t="n">
         <v>3546.33</v>
       </c>
+      <c r="I5" s="21" t="n">
+        <v>1749.36</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Profit Factor</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="8" t="n">
         <v>1.41</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="8" t="n">
         <v>1.25</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="8" t="n">
         <v>1.24</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="8" t="n">
         <v>1.36</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="8" t="n">
         <v>2.17</v>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="8" t="n">
         <v>1.2215</v>
       </c>
-      <c r="H6" s="15" t="n">
+      <c r="H6" s="8" t="n">
         <v>1.27</v>
       </c>
+      <c r="I6" s="22" t="n">
+        <v>2.638</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Total Trades</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="9" t="n">
         <v>560</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="9" t="n">
         <v>629</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="9" t="n">
         <v>1282</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="9" t="n">
         <v>1602</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="9" t="n">
         <v>373</v>
       </c>
-      <c r="G7" s="16" t="n">
+      <c r="G7" s="9" t="n">
         <v>1781</v>
       </c>
-      <c r="H7" s="16" t="n">
+      <c r="H7" s="9" t="n">
         <v>3068</v>
       </c>
+      <c r="I7" s="23" t="n">
+        <v>381</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Win Rate (%)</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="10" t="n">
         <v>0.4625</v>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="10" t="n">
         <v>0.5659999999999999</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="10" t="n">
         <v>0.5101</v>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="10" t="n">
         <v>0.2672</v>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F8" s="10" t="n">
         <v>0.6783</v>
       </c>
-      <c r="G8" s="17" t="n">
+      <c r="G8" s="10" t="n">
         <v>0.4043</v>
       </c>
-      <c r="H8" s="17" t="n">
+      <c r="H8" s="10" t="n">
         <v>0.675</v>
       </c>
+      <c r="I8" s="24" t="n">
+        <v>0.769</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Loss Rate (%)</t>
         </is>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="10">
         <f>1-B8</f>
         <v/>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="10">
         <f>1-C8</f>
         <v/>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="10">
         <f>1-D8</f>
         <v/>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="10">
         <f>1-E8</f>
         <v/>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="10">
         <f>1-F8</f>
         <v/>
       </c>
-      <c r="G9" s="17">
+      <c r="G9" s="10">
         <f>1-G8</f>
         <v/>
       </c>
-      <c r="H9" s="17">
+      <c r="H9" s="10">
         <f>1-H8</f>
         <v/>
       </c>
+      <c r="I9" s="24">
+        <f>1-I8</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Average Win ($)</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="7" t="n">
         <v>36.58</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="7" t="n">
         <v>23.99</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="7" t="n">
         <v>23.88</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="E10" s="7" t="n">
         <v>44.84</v>
       </c>
-      <c r="F10" s="3" t="n">
+      <c r="F10" s="7" t="n">
         <v>12.07</v>
       </c>
-      <c r="G10" s="14" t="n">
+      <c r="G10" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="H10" s="14" t="n">
+      <c r="H10" s="7" t="n">
         <v>8.08</v>
       </c>
+      <c r="I10" s="21" t="n">
+        <v>9.609999999999999</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Average Loss ($)</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" s="7" t="n">
         <v>-22.36</v>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C11" s="7" t="n">
         <v>-25.1</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D11" s="7" t="n">
         <v>-20.07</v>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="7" t="n">
         <v>-12.06</v>
       </c>
-      <c r="F11" s="3" t="n">
+      <c r="F11" s="7" t="n">
         <v>-11.71</v>
       </c>
-      <c r="G11" s="14" t="n">
+      <c r="G11" s="7" t="n">
         <v>-5</v>
       </c>
-      <c r="H11" s="14" t="n">
+      <c r="H11" s="7" t="n">
         <v>-13.24</v>
       </c>
+      <c r="I11" s="21" t="n">
+        <v>-12.13</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Expectancy per Trade ($)</t>
         </is>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="12">
         <f>B8*B10+B9*B11</f>
         <v/>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="12">
         <f>C8*C10+C9*C11</f>
         <v/>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="12">
         <f>D8*D10+D9*D11</f>
         <v/>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="12">
         <f>E8*E10+E9*E11</f>
         <v/>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="12">
         <f>F8*F10+F9*F11</f>
         <v/>
       </c>
-      <c r="G12" s="18">
+      <c r="G12" s="12">
         <f>G8*G10+G9*G11</f>
         <v/>
       </c>
-      <c r="H12" s="18">
+      <c r="H12" s="12">
         <f>H8*H10+H9*H11</f>
         <v/>
       </c>
+      <c r="I12" s="25">
+        <f>I8*I10+I9*I11</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Balance Drawdown Max ($)</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B13" s="7" t="n">
         <v>317.8</v>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="C13" s="7" t="n">
         <v>327.04</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" s="7" t="n">
         <v>521.33</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E13" s="7" t="n">
         <v>549.1</v>
       </c>
-      <c r="F13" s="3" t="n">
+      <c r="F13" s="7" t="n">
         <v>105.92</v>
       </c>
-      <c r="G13" s="14" t="n">
+      <c r="G13" s="7" t="n">
         <v>132</v>
       </c>
-      <c r="H13" s="14" t="n">
+      <c r="H13" s="7" t="n">
         <v>1857.52</v>
       </c>
+      <c r="I13" s="21" t="n">
+        <v>186.45</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Balance Drawdown Max (%)</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="13" t="n">
         <v>0.0295</v>
       </c>
-      <c r="C14" s="9" t="n">
+      <c r="C14" s="13" t="n">
         <v>0.0298</v>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="13" t="n">
         <v>0.0466</v>
       </c>
-      <c r="E14" s="9" t="n">
+      <c r="E14" s="13" t="n">
         <v>0.0388</v>
       </c>
-      <c r="F14" s="9" t="n">
+      <c r="F14" s="13" t="n">
         <v>0.0101</v>
       </c>
-      <c r="G14" s="19" t="n">
+      <c r="G14" s="13" t="n">
         <v>0.0118</v>
       </c>
-      <c r="H14" s="19" t="n">
+      <c r="H14" s="13" t="n">
         <v>0.1649</v>
       </c>
+      <c r="I14" s="26" t="n">
+        <v>0.0019</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Equity (Floating) Drawdown Max ($)</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B15" s="7" t="n">
         <v>390.38</v>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="C15" s="7" t="n">
         <v>367.97</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="7" t="n">
         <v>537.08</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E15" s="7" t="n">
         <v>581.59</v>
       </c>
-      <c r="F15" s="3" t="n">
+      <c r="F15" s="7" t="n">
         <v>117.73</v>
       </c>
-      <c r="G15" s="14" t="n">
+      <c r="G15" s="7" t="n">
         <v>132</v>
       </c>
-      <c r="H15" s="14" t="n">
+      <c r="H15" s="7" t="n">
         <v>2523.99</v>
       </c>
+      <c r="I15" s="21" t="n">
+        <v>517.45</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Equity (Floating) Drawdown Max (%)</t>
         </is>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B16" s="13" t="n">
         <v>0.0323</v>
       </c>
-      <c r="C16" s="9" t="n">
+      <c r="C16" s="13" t="n">
         <v>0.0335</v>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="13" t="n">
         <v>0.048</v>
       </c>
-      <c r="E16" s="9" t="n">
+      <c r="E16" s="13" t="n">
         <v>0.0579</v>
       </c>
-      <c r="F16" s="9" t="n">
+      <c r="F16" s="13" t="n">
         <v>0.0106</v>
       </c>
-      <c r="G16" s="19" t="n">
+      <c r="G16" s="13" t="n">
         <v>0.0118</v>
       </c>
-      <c r="H16" s="19" t="n">
+      <c r="H16" s="13" t="n">
         <v>0.224</v>
       </c>
+      <c r="I16" s="26" t="n">
+        <v>0.0052</v>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Backtest Days</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B17" s="9" t="n">
         <v>982</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="9" t="n">
         <v>982</v>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D17" s="9" t="n">
         <v>982</v>
       </c>
-      <c r="E17" s="5" t="n">
+      <c r="E17" s="9" t="n">
         <v>982</v>
       </c>
-      <c r="F17" s="5" t="n">
+      <c r="F17" s="9" t="n">
         <v>982</v>
       </c>
-      <c r="G17" s="16" t="n">
+      <c r="G17" s="9" t="n">
         <v>982</v>
       </c>
-      <c r="H17" s="16" t="n">
+      <c r="H17" s="9" t="n">
         <v>984</v>
       </c>
+      <c r="I17" s="23" t="n">
+        <v>2079</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>Avg $/Day</t>
         </is>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="12">
         <f>B5/B17</f>
         <v/>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="12">
         <f>C5/C17</f>
         <v/>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="12">
         <f>D5/D17</f>
         <v/>
       </c>
-      <c r="E18" s="8">
+      <c r="E18" s="12">
         <f>E5/E17</f>
         <v/>
       </c>
-      <c r="F18" s="8">
+      <c r="F18" s="12">
         <f>F5/F17</f>
         <v/>
       </c>
-      <c r="G18" s="18">
+      <c r="G18" s="12">
         <f>G5/G17</f>
         <v/>
       </c>
-      <c r="H18" s="18">
+      <c r="H18" s="12">
         <f>H5/H17</f>
         <v/>
       </c>
+      <c r="I18" s="25">
+        <f>I5/I17</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Avg Trades/Day</t>
         </is>
       </c>
-      <c r="B19" s="4">
+      <c r="B19" s="8">
         <f>B7/B17</f>
         <v/>
       </c>
-      <c r="C19" s="4">
+      <c r="C19" s="8">
         <f>C7/C17</f>
         <v/>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="8">
         <f>D7/D17</f>
         <v/>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="8">
         <f>E7/E17</f>
         <v/>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="8">
         <f>F7/F17</f>
         <v/>
       </c>
-      <c r="G19" s="15">
+      <c r="G19" s="8">
         <f>G7/G17</f>
         <v/>
       </c>
-      <c r="H19" s="15">
+      <c r="H19" s="8">
         <f>H7/H17</f>
         <v/>
       </c>
-    </row>
-    <row r="22" ht="15.5" customHeight="1" s="21">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="I19" s="22">
+        <f>I7/I17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="15.5" customHeight="1" s="18">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>Best (Default) Config per Bot</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+    <row r="23" ht="31" customHeight="1" s="18">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>RegimeBot (H1)</t>
         </is>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>H1 Ratchet</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="D23" s="14" t="inlineStr">
         <is>
           <t>M30 Ratchet</t>
         </is>
       </c>
-      <c r="D23" s="11" t="inlineStr">
+      <c r="E23" s="14" t="inlineStr">
         <is>
           <t>M15 Scalper</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="F23" s="14" t="inlineStr">
         <is>
           <t>M5 Scalper</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" s="14" t="inlineStr">
         <is>
           <t>EMA/BB Cross (M5)</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H23" s="14" t="inlineStr">
         <is>
           <t>BB (6TF, EMA-chase)</t>
         </is>
       </c>
-    </row>
-    <row r="24" ht="23" customHeight="1" s="21">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>preBB v6 (%K, 4TF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="77.5" customHeight="1" s="18">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>ADX Trend/Range thresh: 24 / 14</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr">
         <is>
           <t>SL 25 / ratchet-trailing TP (fib, min dist 20)</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>Same engine/file as H1 Ratchet, M30 timeframe slot</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>SL 12 / TP 45 fixed</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="F24" s="15" t="inlineStr">
         <is>
           <t>No-SL on the 1st trade of the day; TP 15 fixed</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" s="15" t="inlineStr">
         <is>
           <t>EMA(20) crosses BB(20,2.0) mid -&gt; instant market buy/sell, SL 5 / TP 9 (real price distance, broker-independent)</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H24" s="15" t="inlineStr">
         <is>
           <t>BB(20,2.0) x6 TF: M1/M5/M15/M30/H1 (H4 orig off)</t>
         </is>
       </c>
-    </row>
-    <row r="25" ht="34.5" customHeight="1" s="21">
-      <c r="A25" s="12" t="inlineStr">
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>K_Threshold_Pct=0.55 (% of band price, NOT fixed $ -- scales with gold's price level)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34.5" customHeight="1" s="18">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>Momentum buy/sell thresh: 1.5 / 2.0</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="C25" s="15" t="inlineStr">
         <is>
           <t>Trailing: start 25, lock 10, gap-trigger 3, SL/TP step 1.5/1.0</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="D25" s="15" t="inlineStr">
         <is>
           <t>SL 20, ADX floor 20 (own values; shares MA50/Vol/hour/max-signal settings above)</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="E25" s="15" t="inlineStr">
         <is>
           <t>MA50-Daily filter: ON</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="F25" s="15" t="inlineStr">
         <is>
           <t>Hard-close after 4 hours if TP not hit</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" s="15" t="inlineStr">
         <is>
           <t>Hour filter: blocks server hours 10, 18, 19</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H25" s="15" t="inlineStr">
         <is>
           <t>THS/THB: instant market, bid/ask vs band, TP=band, thr=4</t>
         </is>
       </c>
-    </row>
-    <row r="26" ht="34.5" customHeight="1" s="21">
-      <c r="A26" s="12" t="inlineStr">
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Per-TF ChaseFraction: M5=0.6, M15=0.5, M30=0.75, H1=0.5 (TP re-pegs toward close each bar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34.5" customHeight="1" s="18">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>XAU/XAG ratio signal: sell 0.014, buy 0.010, gate 20-bar/0.02</t>
         </is>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="C26" s="15" t="inlineStr">
         <is>
           <t>MA50-Daily filter: ON</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>Ratchet trailing, MA50, Vol-spike, hour filter, max 3 signals/day: same as H1</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>ADX floor 24, ceiling 40: ON</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="F26" s="15" t="inlineStr">
         <is>
           <t>Min candle body &gt;= 5 points</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="15" t="inlineStr">
         <is>
           <t>Minute-of-hour filter: buy only at :05/:40/:50, sell only at :40</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H26" s="15" t="inlineStr">
         <is>
           <t>THS2/THB2 addon: limit at bar wick, TP=band, cancel after 1 bar</t>
         </is>
       </c>
-    </row>
-    <row r="27" ht="34.5" customHeight="1" s="21">
-      <c r="A27" s="12" t="inlineStr">
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>InpMaxBarsHold=0 (unbounded) -- TP chase has no hard time cap, can hold through weekends</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="34.5" customHeight="1" s="18">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>MA50-Daily trend filter: ON</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="C27" s="15" t="inlineStr">
         <is>
           <t>ADX floor 24, ceiling 40 + reverse-on-ceiling: ON</t>
         </is>
       </c>
-      <c r="C27" s="12" t="inlineStr">
+      <c r="D27" s="15" t="inlineStr">
         <is>
           <t>Fixed lot 0.01</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="E27" s="15" t="inlineStr">
         <is>
           <t>Hour filter: blocks server hours 7, 22</t>
         </is>
       </c>
-      <c r="E27" s="12" t="inlineStr">
+      <c r="F27" s="15" t="inlineStr">
         <is>
           <t>Level-rejection filter: Fib 38.2/50/61.8% + Day High/Low, proximity 8 (OR logic)</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="15" t="inlineStr">
         <is>
           <t>No trend/volatility/pre-cross filter (tested, none improved results)</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" s="15" t="inlineStr">
         <is>
           <t>TP re-pegs every bar (EMA frac=0.6 orig, 0.667 addon), no fixed SL</t>
         </is>
       </c>
-    </row>
-    <row r="28" ht="34.5" customHeight="1" s="21">
-      <c r="A28" s="12" t="inlineStr">
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Signal: bar0.high-upperBand&gt;thr -&gt; instant SELL TP=band / bar0.low&lt;lowerBand-thr -&gt; instant BUY TP=band</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34.5" customHeight="1" s="18">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>Volatility-spike filter: ON</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="C28" s="15" t="inlineStr">
         <is>
           <t>Volatility-spike filter: ON</t>
         </is>
       </c>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="12" t="inlineStr">
+      <c r="D28" s="15" t="n"/>
+      <c r="E28" s="15" t="inlineStr">
         <is>
           <t>Max 3 signals/day</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="F28" s="15" t="inlineStr">
         <is>
           <t>Max 2 signals/day, 2nd only allowed as an immediate streak-continuation (bypass)</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="15" t="inlineStr">
         <is>
           <t>Max concurrent M5 positions: unlimited (0)</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H28" s="15" t="inlineStr">
         <is>
           <t>Addon requires wick AND close both clear threshold (filters noise)</t>
         </is>
       </c>
-    </row>
-    <row r="29" ht="34.5" customHeight="1" s="21">
-      <c r="A29" s="12" t="inlineStr">
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Addon (THS2/THB2 limit-fade) removed; M1/H4 removed, now M5/M15/M30/H1 only</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="34.5" customHeight="1" s="18">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>News filter (NFP/FOMC/CPI, +/-30min): ON</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="C29" s="15" t="inlineStr">
         <is>
           <t>Hour filter: blocks server hours 7, 22</t>
         </is>
       </c>
-      <c r="C29" s="12" t="n"/>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="D29" s="15" t="n"/>
+      <c r="E29" s="15" t="inlineStr">
         <is>
           <t>Fixed lot 0.01</t>
         </is>
       </c>
-      <c r="E29" s="12" t="inlineStr">
+      <c r="F29" s="15" t="inlineStr">
         <is>
           <t>2nd trade shares the 1st trade's TP; once confirmed, both share SL = midpoint(entry1, entry2)</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="15" t="inlineStr">
         <is>
           <t>Fixed lot 0.01</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H29" s="15" t="inlineStr">
         <is>
           <t>Per-TF isolate switches: H4 orig off, M1 addon off (both underperformed)</t>
         </is>
       </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Fixed lot 0.01, all 4 TF run concurrently, own magic number each</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="31" customHeight="1" s="18">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>Max-DD auto-shutoff: 15%</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr">
         <is>
           <t>Max 3 signals/day</t>
         </is>
       </c>
-      <c r="C30" s="12" t="n"/>
-      <c r="D30" s="12" t="n"/>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="D30" s="15" t="n"/>
+      <c r="E30" s="15" t="n"/>
+      <c r="F30" s="15" t="inlineStr">
         <is>
           <t>MA50-Daily filter: ON</t>
         </is>
       </c>
-    </row>
-    <row r="31" ht="23" customHeight="1" s="21">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="G30" s="15" t="n"/>
+      <c r="H30" s="15" t="n"/>
+    </row>
+    <row r="31" ht="62" customHeight="1" s="18">
+      <c r="B31" s="15" t="inlineStr">
         <is>
           <t>Fixed lot 0.01 (risk-% sizing OFF - tested unstable, causes runaway DD)</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="C31" s="15" t="inlineStr">
         <is>
           <t>Fixed lot 0.01</t>
         </is>
       </c>
-      <c r="C31" s="12" t="n"/>
-      <c r="D31" s="12" t="n"/>
-      <c r="E31" s="12" t="inlineStr">
+      <c r="D31" s="15" t="n"/>
+      <c r="E31" s="15" t="n"/>
+      <c r="F31" s="15" t="inlineStr">
         <is>
           <t>Fixed lot 0.01</t>
         </is>
       </c>
+      <c r="G31" s="15" t="n"/>
+      <c r="H31" s="15" t="n"/>
     </row>
     <row r="32"/>
     <row r="33"/>
     <row r="34">
-      <c r="A34" s="23" t="inlineStr">
+      <c r="A34" s="16" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
@@ -1403,37 +1519,65 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="20" t="inlineStr">
         <is>
           <t>BB.mq5: no fixed TP/SL -- TP chases toward latest close each bar (EMA),</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="20" t="inlineStr">
         <is>
           <t>closing the unbounded-loss failure mode a static TP had on trends.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="20" t="inlineStr">
         <is>
           <t>Validated via 70/30 split + 3-window walk-forward + permutation test</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="20" t="inlineStr">
         <is>
           <t>(drawdown clusters on correlated multi-TF entries during shared moves,</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="20" t="inlineStr">
         <is>
           <t>confirmed structural via permutation, not a fragile-edge symptom).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>preBB v6: validated via real MT5 Strategy Tester (Model=2 OHLC, 2021.01-2026.09, ~5.7yr) with permutation test (2000 shuffles, real maxDD at 12th percentile -- no unlucky clustering), 70/30 split (test PF 2.91 &gt; train PF 2.53, holds cleanly), and a REAL walk-forward (re-optimize K on a 2yr train window, test the next 6mo blind) -- walk-forward found K itself is unstable across windows (hits grid edges), a genuine caveat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>CRITICAL CAVEAT: 83% of total net profit ($1451 of $1749) comes from a single 4-month window (2026 Jan-Apr) -- outside that window several quarters are net losers (2022 Sep-Dec PF 0.28, 2023 Jan-Apr PF 0.27). Same regime-concentration risk pattern as RegimeBot's bull/non-bull finding. NOT yet forward-tested live/demo -- do not treat as sale-ready until a live tracking period confirms the backtest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Repaint check done: entry signal reads the BB band value at shift=0 (forming bar, matches design intent 'instant at bar open') vs shift=1 (closed bar) tested side by side -- shift0 (wired) has a cleaner permutation/DD profile (fewer, higher-conviction trades); shift1 trades 3x more often with more net $ but worse risk (higher DD, permutation shows some correlated clustering at 86th percentile). Whether shift0's band value is truly live-actionable at the exact instant of bar-open (vs a backtest simplification) is unresolved without a live/forward test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Per-TF K% re-swept separately (isolated, 0.20-1.80 range): all 4 TF individually prefer higher K (~0.9-1.2%) by PF, but those samples are tiny (10-27 trades/5.7yr) and 64-79% concentrated in 2026 -- same overfitting pattern, not trusted. Global K=0.55 (shared across all TF, the original design constraint) remains the better-supported choice by net profit and sample robustness, even though it's not the per-TF PF-optimal point.</t>
         </is>
       </c>
     </row>
@@ -1445,10 +1589,11 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A37:F37"/>
     <mergeCell ref="A40:F40"/>
+    <mergeCell ref="A35:F35"/>
     <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A35:F35"/>
     <mergeCell ref="A39:F39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add preBB_Intrabar (intrabar-fire variant) to bot comparison report
New EA that fires the instant the BB threshold crosses intrabar instead of
waiting for bar close, with per-TF K/RSI(14)-confirmation gating. Validated
with permutation test, 70/30 split, and a real per-window walk-forward.

Nets more $ in-sample than preBB v6 but with a worse permutation-test profile
(88-92nd percentile vs preBB v6's 12th, confirming real correlated-loss
clustering) and the walk-forward found two real losing windows in 2023
before turning profitable from 2024 onward, with 89% of total profit
concentrated in a single 2026H1 window. preBB v6 remains the better-supported
choice between the two pending live forward-testing of either.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/XAUUSD_Bot_Comparison.xlsx
+++ b/reports/XAUUSD_Bot_Comparison.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="27580" windowHeight="17740" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="360" windowWidth="38620" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bot Comparison" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -132,12 +132,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -167,11 +164,12 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -543,1011 +541,1107 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="33.1796875" customWidth="1" style="18" min="1" max="1"/>
-    <col width="28" customWidth="1" style="18" min="2" max="5"/>
-    <col width="16" customWidth="1" style="18" min="6" max="6"/>
-    <col width="26.7265625" customWidth="1" style="18" min="7" max="7"/>
-    <col width="22.81640625" customWidth="1" style="18" min="8" max="8"/>
+    <col width="33.1796875" customWidth="1" style="15" min="1" max="1"/>
+    <col width="28" customWidth="1" style="15" min="2" max="5"/>
+    <col width="16" customWidth="1" style="15" min="6" max="6"/>
+    <col width="26.7265625" customWidth="1" style="15" min="7" max="7"/>
+    <col width="22.81640625" customWidth="1" style="15" min="8" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="18">
-      <c r="A1" s="4" t="inlineStr">
+    <row r="1" ht="18" customHeight="1" s="15">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>XAUUSD Bot Portfolio - Backtest Comparison</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Backtest period: 2024.01.01 - 2026.09.09 (982 days) - Real MT5 Strategy Tester, fixed lot 0.01, Model=Open prices (Model=1)</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1" s="18">
-      <c r="A4" s="5" t="inlineStr">
+    <row r="4" ht="28" customHeight="1" s="15">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>RegimeBot (H1)</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>H1 Ratchet</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>M30 Ratchet</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>M15 Scalper</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>M5 Scalper</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>EMA/BB Cross (M5)</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>BB (6TF, EMA-chase)</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>preBB v6 (%K, 4TF)</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>preBB Intrabar (%K, RSI-gated)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Total Net Profit ($)</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="4" t="n">
         <v>2744.24</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="4" t="n">
         <v>1689.42</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="4" t="n">
         <v>3015.39</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="4" t="n">
         <v>5035.78</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="F5" s="4" t="n">
         <v>1647.24</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="G5" s="4" t="n">
         <v>1175</v>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="H5" s="4" t="n">
         <v>3546.33</v>
       </c>
-      <c r="I5" s="21" t="n">
+      <c r="I5" s="4" t="n">
         <v>1749.36</v>
       </c>
+      <c r="J5" s="19" t="n">
+        <v>2814.15</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Profit Factor</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="5" t="n">
         <v>1.41</v>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="5" t="n">
         <v>1.25</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="5" t="n">
         <v>1.24</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="5" t="n">
         <v>1.36</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="5" t="n">
         <v>2.17</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="5" t="n">
         <v>1.2215</v>
       </c>
-      <c r="H6" s="8" t="n">
+      <c r="H6" s="5" t="n">
         <v>1.27</v>
       </c>
-      <c r="I6" s="22" t="n">
+      <c r="I6" s="5" t="n">
         <v>2.638</v>
       </c>
+      <c r="J6" s="20" t="n">
+        <v>1.854</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Total Trades</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="6" t="n">
         <v>560</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="6" t="n">
         <v>629</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="6" t="n">
         <v>1282</v>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="E7" s="6" t="n">
         <v>1602</v>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F7" s="6" t="n">
         <v>373</v>
       </c>
-      <c r="G7" s="9" t="n">
+      <c r="G7" s="6" t="n">
         <v>1781</v>
       </c>
-      <c r="H7" s="9" t="n">
+      <c r="H7" s="6" t="n">
         <v>3068</v>
       </c>
-      <c r="I7" s="23" t="n">
+      <c r="I7" s="6" t="n">
         <v>381</v>
       </c>
+      <c r="J7" s="21" t="n">
+        <v>709</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Win Rate (%)</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="7" t="n">
         <v>0.4625</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="7" t="n">
         <v>0.5659999999999999</v>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D8" s="7" t="n">
         <v>0.5101</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="7" t="n">
         <v>0.2672</v>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" s="7" t="n">
         <v>0.6783</v>
       </c>
-      <c r="G8" s="10" t="n">
+      <c r="G8" s="7" t="n">
         <v>0.4043</v>
       </c>
-      <c r="H8" s="10" t="n">
+      <c r="H8" s="7" t="n">
         <v>0.675</v>
       </c>
-      <c r="I8" s="24" t="n">
+      <c r="I8" s="7" t="n">
         <v>0.769</v>
       </c>
+      <c r="J8" s="22" t="n">
+        <v>0.6870000000000001</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Loss Rate (%)</t>
         </is>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="7">
         <f>1-B8</f>
         <v/>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="7">
         <f>1-C8</f>
         <v/>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="7">
         <f>1-D8</f>
         <v/>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="7">
         <f>1-E8</f>
         <v/>
       </c>
-      <c r="F9" s="10">
+      <c r="F9" s="7">
         <f>1-F8</f>
         <v/>
       </c>
-      <c r="G9" s="10">
+      <c r="G9" s="7">
         <f>1-G8</f>
         <v/>
       </c>
-      <c r="H9" s="10">
+      <c r="H9" s="7">
         <f>1-H8</f>
         <v/>
       </c>
-      <c r="I9" s="24">
+      <c r="I9" s="7">
         <f>1-I8</f>
         <v/>
       </c>
+      <c r="J9" s="22">
+        <f>1-J8</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Average Win ($)</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="4" t="n">
         <v>36.58</v>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="4" t="n">
         <v>23.99</v>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="4" t="n">
         <v>23.88</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E10" s="4" t="n">
         <v>44.84</v>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="F10" s="4" t="n">
         <v>12.07</v>
       </c>
-      <c r="G10" s="7" t="n">
+      <c r="G10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="H10" s="4" t="n">
         <v>8.08</v>
       </c>
-      <c r="I10" s="21" t="n">
+      <c r="I10" s="4" t="n">
         <v>9.609999999999999</v>
       </c>
+      <c r="J10" s="19" t="n">
+        <v>12.54</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Average Loss ($)</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="4" t="n">
         <v>-22.36</v>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="4" t="n">
         <v>-25.1</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="4" t="n">
         <v>-20.07</v>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E11" s="4" t="n">
         <v>-12.06</v>
       </c>
-      <c r="F11" s="7" t="n">
+      <c r="F11" s="4" t="n">
         <v>-11.71</v>
       </c>
-      <c r="G11" s="7" t="n">
+      <c r="G11" s="4" t="n">
         <v>-5</v>
       </c>
-      <c r="H11" s="7" t="n">
+      <c r="H11" s="4" t="n">
         <v>-13.24</v>
       </c>
-      <c r="I11" s="21" t="n">
+      <c r="I11" s="4" t="n">
         <v>-12.13</v>
       </c>
+      <c r="J11" s="19" t="n">
+        <v>-14.84</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Expectancy per Trade ($)</t>
         </is>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="9">
         <f>B8*B10+B9*B11</f>
         <v/>
       </c>
-      <c r="C12" s="12">
+      <c r="C12" s="9">
         <f>C8*C10+C9*C11</f>
         <v/>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="9">
         <f>D8*D10+D9*D11</f>
         <v/>
       </c>
-      <c r="E12" s="12">
+      <c r="E12" s="9">
         <f>E8*E10+E9*E11</f>
         <v/>
       </c>
-      <c r="F12" s="12">
+      <c r="F12" s="9">
         <f>F8*F10+F9*F11</f>
         <v/>
       </c>
-      <c r="G12" s="12">
+      <c r="G12" s="9">
         <f>G8*G10+G9*G11</f>
         <v/>
       </c>
-      <c r="H12" s="12">
+      <c r="H12" s="9">
         <f>H8*H10+H9*H11</f>
         <v/>
       </c>
-      <c r="I12" s="25">
+      <c r="I12" s="9">
         <f>I8*I10+I9*I11</f>
         <v/>
       </c>
+      <c r="J12" s="23">
+        <f>J8*J10+J9*J11</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Balance Drawdown Max ($)</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="4" t="n">
         <v>317.8</v>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="4" t="n">
         <v>327.04</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="4" t="n">
         <v>521.33</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="E13" s="4" t="n">
         <v>549.1</v>
       </c>
-      <c r="F13" s="7" t="n">
+      <c r="F13" s="4" t="n">
         <v>105.92</v>
       </c>
-      <c r="G13" s="7" t="n">
+      <c r="G13" s="4" t="n">
         <v>132</v>
       </c>
-      <c r="H13" s="7" t="n">
+      <c r="H13" s="4" t="n">
         <v>1857.52</v>
       </c>
-      <c r="I13" s="21" t="n">
+      <c r="I13" s="4" t="n">
         <v>186.45</v>
       </c>
+      <c r="J13" s="19" t="n">
+        <v>341.54</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Balance Drawdown Max (%)</t>
         </is>
       </c>
-      <c r="B14" s="13" t="n">
+      <c r="B14" s="10" t="n">
         <v>0.0295</v>
       </c>
-      <c r="C14" s="13" t="n">
+      <c r="C14" s="10" t="n">
         <v>0.0298</v>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="10" t="n">
         <v>0.0466</v>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E14" s="10" t="n">
         <v>0.0388</v>
       </c>
-      <c r="F14" s="13" t="n">
+      <c r="F14" s="10" t="n">
         <v>0.0101</v>
       </c>
-      <c r="G14" s="13" t="n">
+      <c r="G14" s="10" t="n">
         <v>0.0118</v>
       </c>
-      <c r="H14" s="13" t="n">
+      <c r="H14" s="10" t="n">
         <v>0.1649</v>
       </c>
-      <c r="I14" s="26" t="n">
+      <c r="I14" s="10" t="n">
         <v>0.0019</v>
       </c>
+      <c r="J14" s="24" t="n">
+        <v>0.00331</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Equity (Floating) Drawdown Max ($)</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="4" t="n">
         <v>390.38</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="4" t="n">
         <v>367.97</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="4" t="n">
         <v>537.08</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="E15" s="4" t="n">
         <v>581.59</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="F15" s="4" t="n">
         <v>117.73</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="G15" s="4" t="n">
         <v>132</v>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="H15" s="4" t="n">
         <v>2523.99</v>
       </c>
-      <c r="I15" s="21" t="n">
+      <c r="I15" s="4" t="n">
         <v>517.45</v>
       </c>
+      <c r="J15" s="19" t="n">
+        <v>1007.42</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Equity (Floating) Drawdown Max (%)</t>
         </is>
       </c>
-      <c r="B16" s="13" t="n">
+      <c r="B16" s="10" t="n">
         <v>0.0323</v>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C16" s="10" t="n">
         <v>0.0335</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D16" s="10" t="n">
         <v>0.048</v>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E16" s="10" t="n">
         <v>0.0579</v>
       </c>
-      <c r="F16" s="13" t="n">
+      <c r="F16" s="10" t="n">
         <v>0.0106</v>
       </c>
-      <c r="G16" s="13" t="n">
+      <c r="G16" s="10" t="n">
         <v>0.0118</v>
       </c>
-      <c r="H16" s="13" t="n">
+      <c r="H16" s="10" t="n">
         <v>0.224</v>
       </c>
-      <c r="I16" s="26" t="n">
+      <c r="I16" s="10" t="n">
         <v>0.0052</v>
       </c>
+      <c r="J16" s="24" t="n">
+        <v>0.01002</v>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Backtest Days</t>
         </is>
       </c>
-      <c r="B17" s="9" t="n">
+      <c r="B17" s="6" t="n">
         <v>982</v>
       </c>
-      <c r="C17" s="9" t="n">
+      <c r="C17" s="6" t="n">
         <v>982</v>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="6" t="n">
         <v>982</v>
       </c>
-      <c r="E17" s="9" t="n">
+      <c r="E17" s="6" t="n">
         <v>982</v>
       </c>
-      <c r="F17" s="9" t="n">
+      <c r="F17" s="6" t="n">
         <v>982</v>
       </c>
-      <c r="G17" s="9" t="n">
+      <c r="G17" s="6" t="n">
         <v>982</v>
       </c>
-      <c r="H17" s="9" t="n">
+      <c r="H17" s="6" t="n">
         <v>984</v>
       </c>
-      <c r="I17" s="23" t="n">
+      <c r="I17" s="6" t="n">
         <v>2079</v>
       </c>
+      <c r="J17" s="21" t="n">
+        <v>2079</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Avg $/Day</t>
         </is>
       </c>
-      <c r="B18" s="12">
+      <c r="B18" s="9">
         <f>B5/B17</f>
         <v/>
       </c>
-      <c r="C18" s="12">
+      <c r="C18" s="9">
         <f>C5/C17</f>
         <v/>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="9">
         <f>D5/D17</f>
         <v/>
       </c>
-      <c r="E18" s="12">
+      <c r="E18" s="9">
         <f>E5/E17</f>
         <v/>
       </c>
-      <c r="F18" s="12">
+      <c r="F18" s="9">
         <f>F5/F17</f>
         <v/>
       </c>
-      <c r="G18" s="12">
+      <c r="G18" s="9">
         <f>G5/G17</f>
         <v/>
       </c>
-      <c r="H18" s="12">
+      <c r="H18" s="9">
         <f>H5/H17</f>
         <v/>
       </c>
-      <c r="I18" s="25">
+      <c r="I18" s="9">
         <f>I5/I17</f>
         <v/>
       </c>
+      <c r="J18" s="23">
+        <f>J5/J17</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Avg Trades/Day</t>
         </is>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="5">
         <f>B7/B17</f>
         <v/>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="5">
         <f>C7/C17</f>
         <v/>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="5">
         <f>D7/D17</f>
         <v/>
       </c>
-      <c r="E19" s="8">
+      <c r="E19" s="5">
         <f>E7/E17</f>
         <v/>
       </c>
-      <c r="F19" s="8">
+      <c r="F19" s="5">
         <f>F7/F17</f>
         <v/>
       </c>
-      <c r="G19" s="8">
+      <c r="G19" s="5">
         <f>G7/G17</f>
         <v/>
       </c>
-      <c r="H19" s="8">
+      <c r="H19" s="5">
         <f>H7/H17</f>
         <v/>
       </c>
-      <c r="I19" s="22">
+      <c r="I19" s="5">
         <f>I7/I17</f>
         <v/>
       </c>
-    </row>
-    <row r="22" ht="15.5" customHeight="1" s="18">
+      <c r="J19" s="20">
+        <f>J7/J17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="15.5" customHeight="1" s="15">
       <c r="A22" s="1" t="inlineStr">
         <is>
           <t>Best (Default) Config per Bot</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="31" customHeight="1" s="18">
-      <c r="B23" s="14" t="inlineStr">
+    <row r="23" ht="31" customHeight="1" s="15">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>RegimeBot (H1)</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>H1 Ratchet</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>M30 Ratchet</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E23" s="11" t="inlineStr">
         <is>
           <t>M15 Scalper</t>
         </is>
       </c>
-      <c r="F23" s="14" t="inlineStr">
+      <c r="F23" s="11" t="inlineStr">
         <is>
           <t>M5 Scalper</t>
         </is>
       </c>
-      <c r="G23" s="14" t="inlineStr">
+      <c r="G23" s="11" t="inlineStr">
         <is>
           <t>EMA/BB Cross (M5)</t>
         </is>
       </c>
-      <c r="H23" s="14" t="inlineStr">
+      <c r="H23" s="11" t="inlineStr">
         <is>
           <t>BB (6TF, EMA-chase)</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I23" s="11" t="inlineStr">
         <is>
           <t>preBB v6 (%K, 4TF)</t>
         </is>
       </c>
-    </row>
-    <row r="24" ht="77.5" customHeight="1" s="18">
-      <c r="B24" s="15" t="inlineStr">
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>preBB Intrabar (%K, RSI-gated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="77.5" customHeight="1" s="15">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>ADX Trend/Range thresh: 24 / 14</t>
         </is>
       </c>
-      <c r="C24" s="15" t="inlineStr">
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>SL 25 / ratchet-trailing TP (fib, min dist 20)</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>Same engine/file as H1 Ratchet, M30 timeframe slot</t>
         </is>
       </c>
-      <c r="E24" s="15" t="inlineStr">
+      <c r="E24" s="12" t="inlineStr">
         <is>
           <t>SL 12 / TP 45 fixed</t>
         </is>
       </c>
-      <c r="F24" s="15" t="inlineStr">
+      <c r="F24" s="12" t="inlineStr">
         <is>
           <t>No-SL on the 1st trade of the day; TP 15 fixed</t>
         </is>
       </c>
-      <c r="G24" s="15" t="inlineStr">
+      <c r="G24" s="12" t="inlineStr">
         <is>
           <t>EMA(20) crosses BB(20,2.0) mid -&gt; instant market buy/sell, SL 5 / TP 9 (real price distance, broker-independent)</t>
         </is>
       </c>
-      <c r="H24" s="15" t="inlineStr">
+      <c r="H24" s="12" t="inlineStr">
         <is>
           <t>BB(20,2.0) x6 TF: M1/M5/M15/M30/H1 (H4 orig off)</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I24" s="12" t="inlineStr">
         <is>
           <t>K_Threshold_Pct=0.55 (% of band price, NOT fixed $ -- scales with gold's price level)</t>
         </is>
       </c>
-    </row>
-    <row r="25" ht="34.5" customHeight="1" s="18">
-      <c r="B25" s="15" t="inlineStr">
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Fires INTRABAR (every tick), not at bar close: compares the still-forming bar's running high/low vs the LIVE band value, fires the instant K threshold is crossed. TP = live band value at fire instant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34.5" customHeight="1" s="15">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>Momentum buy/sell thresh: 1.5 / 2.0</t>
         </is>
       </c>
-      <c r="C25" s="15" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>Trailing: start 25, lock 10, gap-trigger 3, SL/TP step 1.5/1.0</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>SL 20, ADX floor 20 (own values; shares MA50/Vol/hour/max-signal settings above)</t>
         </is>
       </c>
-      <c r="E25" s="15" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>MA50-Daily filter: ON</t>
         </is>
       </c>
-      <c r="F25" s="15" t="inlineStr">
+      <c r="F25" s="12" t="inlineStr">
         <is>
           <t>Hard-close after 4 hours if TP not hit</t>
         </is>
       </c>
-      <c r="G25" s="15" t="inlineStr">
+      <c r="G25" s="12" t="inlineStr">
         <is>
           <t>Hour filter: blocks server hours 10, 18, 19</t>
         </is>
       </c>
-      <c r="H25" s="15" t="inlineStr">
+      <c r="H25" s="12" t="inlineStr">
         <is>
           <t>THS/THB: instant market, bid/ask vs band, TP=band, thr=4</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I25" s="12" t="inlineStr">
         <is>
           <t>Per-TF ChaseFraction: M5=0.6, M15=0.5, M30=0.75, H1=0.5 (TP re-pegs toward close each bar)</t>
         </is>
       </c>
-    </row>
-    <row r="26" ht="34.5" customHeight="1" s="18">
-      <c r="B26" s="15" t="inlineStr">
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Per-TF K_Threshold_Pct: M5=0.40, M15=0.60, M30=0.60, H1=0.60 (vs preBB v6's single shared K=0.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34.5" customHeight="1" s="15">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>XAU/XAG ratio signal: sell 0.014, buy 0.010, gate 20-bar/0.02</t>
         </is>
       </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
         <is>
           <t>MA50-Daily filter: ON</t>
         </is>
       </c>
-      <c r="D26" s="15" t="inlineStr">
+      <c r="D26" s="12" t="inlineStr">
         <is>
           <t>Ratchet trailing, MA50, Vol-spike, hour filter, max 3 signals/day: same as H1</t>
         </is>
       </c>
-      <c r="E26" s="15" t="inlineStr">
+      <c r="E26" s="12" t="inlineStr">
         <is>
           <t>ADX floor 24, ceiling 40: ON</t>
         </is>
       </c>
-      <c r="F26" s="15" t="inlineStr">
+      <c r="F26" s="12" t="inlineStr">
         <is>
           <t>Min candle body &gt;= 5 points</t>
         </is>
       </c>
-      <c r="G26" s="15" t="inlineStr">
+      <c r="G26" s="12" t="inlineStr">
         <is>
           <t>Minute-of-hour filter: buy only at :05/:40/:50, sell only at :40</t>
         </is>
       </c>
-      <c r="H26" s="15" t="inlineStr">
+      <c r="H26" s="12" t="inlineStr">
         <is>
           <t>THS2/THB2 addon: limit at bar wick, TP=band, cancel after 1 bar</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I26" s="12" t="inlineStr">
         <is>
           <t>InpMaxBarsHold=0 (unbounded) -- TP chase has no hard time cap, can hold through weekends</t>
         </is>
       </c>
-    </row>
-    <row r="27" ht="34.5" customHeight="1" s="18">
-      <c r="B27" s="15" t="inlineStr">
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Per-TF ChaseFraction: M5=0.5, M15=0.5, M30=0.5, H1=0.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="34.5" customHeight="1" s="15">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>MA50-Daily trend filter: ON</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>ADX floor 24, ceiling 40 + reverse-on-ceiling: ON</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>Fixed lot 0.01</t>
         </is>
       </c>
-      <c r="E27" s="15" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>Hour filter: blocks server hours 7, 22</t>
         </is>
       </c>
-      <c r="F27" s="15" t="inlineStr">
+      <c r="F27" s="12" t="inlineStr">
         <is>
           <t>Level-rejection filter: Fib 38.2/50/61.8% + Day High/Low, proximity 8 (OR logic)</t>
         </is>
       </c>
-      <c r="G27" s="15" t="inlineStr">
+      <c r="G27" s="12" t="inlineStr">
         <is>
           <t>No trend/volatility/pre-cross filter (tested, none improved results)</t>
         </is>
       </c>
-      <c r="H27" s="15" t="inlineStr">
+      <c r="H27" s="12" t="inlineStr">
         <is>
           <t>TP re-pegs every bar (EMA frac=0.6 orig, 0.667 addon), no fixed SL</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I27" s="12" t="inlineStr">
         <is>
           <t>Signal: bar0.high-upperBand&gt;thr -&gt; instant SELL TP=band / bar0.low&lt;lowerBand-thr -&gt; instant BUY TP=band</t>
         </is>
       </c>
-    </row>
-    <row r="28" ht="34.5" customHeight="1" s="18">
-      <c r="B28" s="15" t="inlineStr">
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>RSI(14) confirmation gate (InpUseRSIGate=true): SELL only if RSI(shift1)&gt;=50+X, BUY only if RSI&lt;=50-X, X per TF: M5=0(off), M15=10, M30=5, H1=5. Found the losing zone is mid-momentum RSI 50-70, not extreme overbought/oversold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34.5" customHeight="1" s="15">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>Volatility-spike filter: ON</t>
         </is>
       </c>
-      <c r="C28" s="15" t="inlineStr">
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>Volatility-spike filter: ON</t>
         </is>
       </c>
-      <c r="D28" s="15" t="n"/>
-      <c r="E28" s="15" t="inlineStr">
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="12" t="inlineStr">
         <is>
           <t>Max 3 signals/day</t>
         </is>
       </c>
-      <c r="F28" s="15" t="inlineStr">
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>Max 2 signals/day, 2nd only allowed as an immediate streak-continuation (bypass)</t>
         </is>
       </c>
-      <c r="G28" s="15" t="inlineStr">
+      <c r="G28" s="12" t="inlineStr">
         <is>
           <t>Max concurrent M5 positions: unlimited (0)</t>
         </is>
       </c>
-      <c r="H28" s="15" t="inlineStr">
+      <c r="H28" s="12" t="inlineStr">
         <is>
           <t>Addon requires wick AND close both clear threshold (filters noise)</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I28" s="12" t="inlineStr">
         <is>
           <t>Addon (THS2/THB2 limit-fade) removed; M1/H4 removed, now M5/M15/M30/H1 only</t>
         </is>
       </c>
-    </row>
-    <row r="29" ht="34.5" customHeight="1" s="18">
-      <c r="B29" s="15" t="inlineStr">
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Same TP-chase mechanism as preBB v6 (EMA fraction toward close each bar), InpMaxBarsHold=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="34.5" customHeight="1" s="15">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>News filter (NFP/FOMC/CPI, +/-30min): ON</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
         <is>
           <t>Hour filter: blocks server hours 7, 22</t>
         </is>
       </c>
-      <c r="D29" s="15" t="n"/>
-      <c r="E29" s="15" t="inlineStr">
+      <c r="D29" s="12" t="n"/>
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>Fixed lot 0.01</t>
         </is>
       </c>
-      <c r="F29" s="15" t="inlineStr">
+      <c r="F29" s="12" t="inlineStr">
         <is>
           <t>2nd trade shares the 1st trade's TP; once confirmed, both share SL = midpoint(entry1, entry2)</t>
         </is>
       </c>
-      <c r="G29" s="15" t="inlineStr">
+      <c r="G29" s="12" t="inlineStr">
         <is>
           <t>Fixed lot 0.01</t>
         </is>
       </c>
-      <c r="H29" s="15" t="inlineStr">
+      <c r="H29" s="12" t="inlineStr">
         <is>
           <t>Per-TF isolate switches: H4 orig off, M1 addon off (both underperformed)</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I29" s="12" t="inlineStr">
         <is>
           <t>Fixed lot 0.01, all 4 TF run concurrently, own magic number each</t>
         </is>
       </c>
-    </row>
-    <row r="30" ht="31" customHeight="1" s="18">
-      <c r="B30" s="15" t="inlineStr">
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Magics 211005/211015/211030/211060 (different from preBB v6's 111xxx, can run side by side)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="31" customHeight="1" s="15">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Max-DD auto-shutoff: 15%</t>
         </is>
       </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
         <is>
           <t>Max 3 signals/day</t>
         </is>
       </c>
-      <c r="D30" s="15" t="n"/>
-      <c r="E30" s="15" t="n"/>
-      <c r="F30" s="15" t="inlineStr">
+      <c r="D30" s="12" t="n"/>
+      <c r="E30" s="12" t="n"/>
+      <c r="F30" s="12" t="inlineStr">
         <is>
           <t>MA50-Daily filter: ON</t>
         </is>
       </c>
-      <c r="G30" s="15" t="n"/>
-      <c r="H30" s="15" t="n"/>
-    </row>
-    <row r="31" ht="62" customHeight="1" s="18">
-      <c r="B31" s="15" t="inlineStr">
+      <c r="G30" s="12" t="n"/>
+      <c r="H30" s="12" t="n"/>
+      <c r="I30" s="12" t="n"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Fixed lot 0.01, all 4 TF concurrent</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="62" customHeight="1" s="15">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>Fixed lot 0.01 (risk-% sizing OFF - tested unstable, causes runaway DD)</t>
         </is>
       </c>
-      <c r="C31" s="15" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>Fixed lot 0.01</t>
         </is>
       </c>
-      <c r="D31" s="15" t="n"/>
-      <c r="E31" s="15" t="n"/>
-      <c r="F31" s="15" t="inlineStr">
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="12" t="inlineStr">
         <is>
           <t>Fixed lot 0.01</t>
         </is>
       </c>
-      <c r="G31" s="15" t="n"/>
-      <c r="H31" s="15" t="n"/>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="12" t="n"/>
+      <c r="I31" s="12" t="n"/>
     </row>
     <row r="32"/>
     <row r="33"/>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="20" t="inlineStr">
+      <c r="A35" s="14" t="inlineStr">
         <is>
           <t>- Expectancy/Trade = WinRate x AvgWin + LossRate x AvgLoss (AvgLoss is negative). Cross-checked: Expectancy x Trades matches Total Net Profit for every bot.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="20" t="inlineStr">
+      <c r="A36" s="14" t="inlineStr">
         <is>
           <t>- All 5 backtests use the same period, feed, and fixed 0.01 lot for a fair side-by-side comparison.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="20" t="inlineStr">
+      <c r="A37" s="14" t="inlineStr">
         <is>
           <t>- M15/M5 Scalper are two engines inside the same XAUUSD_M15_Scalper.mq5 file, run separately here (one engine enabled at a time) to isolate each engine's own numbers.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="20" t="inlineStr">
+      <c r="A38" s="14" t="inlineStr">
         <is>
           <t>- H1/M30 Ratchet are two engines inside XAUUSD_H1_Ratchet_EA_enhanced_v2.mq5, run separately here for the same reason.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="20" t="inlineStr">
+      <c r="A39" s="14" t="inlineStr">
         <is>
           <t>- Backtest engine: MT5 Strategy Tester, Model=1 (Open prices only) - faster than Every-tick, small variance (a few % on PF/PnL) vs a tick-accurate run should be expected.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="20" t="inlineStr">
+      <c r="A40" s="14" t="inlineStr">
         <is>
           <t>- Naive sum of all 5 bots' Avg $/Day is NOT a validated combined number - running them simultaneously was never tested end-to-end and their signals are not fully independent (measured ~71% day-overlap between H1 and M30 earlier in this project).</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="20" t="inlineStr">
+      <c r="A41" s="14" t="inlineStr">
         <is>
           <t>- EMA/BB Cross (M5) hour/minute filter validated via walk-forward (180d train / 60d test, rolled 60d, 13 folds, rule re-derived fresh each fold): pooled out-of-sample n=1377, WR=37.91%, PF=1.099, net=+$423 -- 10/13 folds profitable. The PF=1.2215/net=$1,175 in the table above is a single in-sample fit on the full period and is optimistic; walk-forward PF~1.10 is the more realistic expectation for live use.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="20" t="inlineStr">
+      <c r="A42" s="14" t="inlineStr">
         <is>
           <t>- A plain 70/30 chronological split (train on first 70%, test blind on last 30%) failed for this same filter (out-of-sample PF=0.970, net=-$51) -- walk-forward's rolling multi-fold average is the more reliable read since a single split is itself high-variance.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="20" t="inlineStr">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>- Permutation test (5000 shuffles of trade outcomes against the fixed hour/minute rule): actual PF=1.2215 exceeded every one of the 5000 random draws (p=0.00000, null median PF=0.980) -- confirms the FIXED rule isn't random noise, but does not by itself prove the rule-discovery process (searching many hour/minute combos) is free of overfitting; the walk-forward result above is what actually tests that.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="20" t="inlineStr">
+      <c r="A44" s="14" t="inlineStr">
         <is>
           <t>BB.mq5: no fixed TP/SL -- TP chases toward latest close each bar (EMA),</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="20" t="inlineStr">
+      <c r="A45" s="14" t="inlineStr">
         <is>
           <t>closing the unbounded-loss failure mode a static TP had on trends.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="20" t="inlineStr">
+      <c r="A46" s="14" t="inlineStr">
         <is>
           <t>Validated via 70/30 split + 3-window walk-forward + permutation test</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="20" t="inlineStr">
+      <c r="A47" s="14" t="inlineStr">
         <is>
           <t>(drawdown clusters on correlated multi-TF entries during shared moves,</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="20" t="inlineStr">
+      <c r="A48" s="14" t="inlineStr">
         <is>
           <t>confirmed structural via permutation, not a fragile-edge symptom).</t>
         </is>
@@ -1578,6 +1672,37 @@
       <c r="A52" t="inlineStr">
         <is>
           <t>Per-TF K% re-swept separately (isolated, 0.20-1.80 range): all 4 TF individually prefer higher K (~0.9-1.2%) by PF, but those samples are tiny (10-27 trades/5.7yr) and 64-79% concentrated in 2026 -- same overfitting pattern, not trusted. Global K=0.55 (shared across all TF, the original design constraint) remains the better-supported choice by net profit and sample robustness, even though it's not the per-TF PF-optimal point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>preBB Intrabar: variant of preBB v6 that fires the instant the band threshold crosses intrabar instead of waiting for bar close, aiming to catch the move earlier. K/RSI-gate strength picked per TF via one-launch MT5 optimization grids, then validated with permutation test (2000 shuffles), 70/30 split, AND a REAL walk-forward (per-TF K+RSI re-optimized on a rolling 2yr train window, tested blind on the next 6mo, 7 windows 2023H1-2026H1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>CRITICAL CAVEAT (worse than preBB v6 on this front): permutation test puts real maxDD at the 88-92nd percentile of 2000 shuffles (preBB v6: 12th) -- real, structural correlated-loss clustering, not random noise. Root-caused to specific TF combos (H1+M15+M30 all holding a position at once) and to entries firing on SELL during mid-momentum RSI (50-70) rather than a true overbought extreme -- price keeps trending against the trade before TP catches up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>CRITICAL CAVEAT: the REAL walk-forward (blind per-window K/RSI selection, no look-ahead) shows 2 consecutive losing windows -- 2023H1 net -7 (PF 0.84) and 2023H2 net -8 (PF 0.77) -- before turning profitable from 2024 onward. 89% of total walk-forward profit (364 of 656) comes from the single 2026H1 window; every other window combined nets only ~92. Same regime-concentration pattern as preBB v6 and RegimeBot, more severe here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>NOT forward-tested live/demo. Given the worse permutation/clustering profile and the confirmed 2023 losing windows, preBB v6 (bar-close) remains the better-supported choice between the two for now -- Intrabar nets more $ in-sample but at a meaningfully worse, walk-forward-confirmed risk profile.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: dump TesterStatistics (DD) to OnTester; add BB M1-blend to comparison report
OnTester now also writes a <name>_stats.csv with net profit, PF, win
rate, avg win/loss, and balance/equity drawdown ($/%) - the deal log
alone can't derive floating-equity DD. Used it to fill in the new
"BB M1-blend (5TF)" column in XAUUSD_Bot_Comparison.xlsx, with a note
that the M1 quadratic-blend edge is regime-dependent (70/30 split +
bootstrap validation was inconsistent between windows).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/XAUUSD_Bot_Comparison.xlsx
+++ b/reports/XAUUSD_Bot_Comparison.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J57"/>
+  <dimension ref="A1:K57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="33.1796875" customWidth="1" style="15" min="1" max="1"/>
@@ -616,6 +616,11 @@
           <t>preBB Intrabar (%K, RSI-gated)</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>BB M1-blend (5TF)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -650,6 +655,9 @@
       <c r="J5" s="19" t="n">
         <v>2814.15</v>
       </c>
+      <c r="K5" s="19" t="n">
+        <v>8206.129999999999</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -684,6 +692,9 @@
       <c r="J6" s="20" t="n">
         <v>1.854</v>
       </c>
+      <c r="K6" s="20" t="n">
+        <v>1.29</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -718,6 +729,9 @@
       <c r="J7" s="21" t="n">
         <v>709</v>
       </c>
+      <c r="K7" s="21" t="n">
+        <v>3520</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -752,6 +766,9 @@
       <c r="J8" s="22" t="n">
         <v>0.6870000000000001</v>
       </c>
+      <c r="K8" s="22" t="n">
+        <v>0.6741</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -795,6 +812,10 @@
         <f>1-J8</f>
         <v/>
       </c>
+      <c r="K9" s="22">
+        <f>1-K8</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -829,6 +850,9 @@
       <c r="J10" s="19" t="n">
         <v>12.54</v>
       </c>
+      <c r="K10" s="19" t="n">
+        <v>15.57</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -863,6 +887,9 @@
       <c r="J11" s="19" t="n">
         <v>-14.84</v>
       </c>
+      <c r="K11" s="19" t="n">
+        <v>-25.05</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -906,6 +933,10 @@
         <f>J8*J10+J9*J11</f>
         <v/>
       </c>
+      <c r="K12" s="23">
+        <f>K8*K10+K9*K11</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -940,6 +971,9 @@
       <c r="J13" s="19" t="n">
         <v>341.54</v>
       </c>
+      <c r="K13" s="19" t="n">
+        <v>3723.76</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -974,6 +1008,9 @@
       <c r="J14" s="24" t="n">
         <v>0.00331</v>
       </c>
+      <c r="K14" s="24" t="n">
+        <v>0.2964</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1008,6 +1045,9 @@
       <c r="J15" s="19" t="n">
         <v>1007.42</v>
       </c>
+      <c r="K15" s="19" t="n">
+        <v>5051.9</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1042,6 +1082,9 @@
       <c r="J16" s="24" t="n">
         <v>0.01002</v>
       </c>
+      <c r="K16" s="24" t="n">
+        <v>0.4019</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1076,6 +1119,9 @@
       <c r="J17" s="21" t="n">
         <v>2079</v>
       </c>
+      <c r="K17" s="21" t="n">
+        <v>996</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -1119,6 +1165,10 @@
         <f>J5/J17</f>
         <v/>
       </c>
+      <c r="K18" s="23">
+        <f>K5/K17</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1162,6 +1212,10 @@
         <f>J7/J17</f>
         <v/>
       </c>
+      <c r="K19" s="20">
+        <f>K7/K17</f>
+        <v/>
+      </c>
     </row>
     <row r="22" ht="15.5" customHeight="1" s="15">
       <c r="A22" s="1" t="inlineStr">
@@ -1216,6 +1270,11 @@
           <t>preBB Intrabar (%K, RSI-gated)</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>BB M1-blend (5TF)</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="77.5" customHeight="1" s="15">
       <c r="B24" s="12" t="inlineStr">
@@ -1263,6 +1322,11 @@
           <t>Fires INTRABAR (every tick), not at bar close: compares the still-forming bar's running high/low vs the LIVE band value, fires the instant K threshold is crossed. TP = live band value at fire instant.</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>BB(20,2.0) x5 TF: M1/M5/M15/M30/H1 (H4 fully off: Enable_H4=false)</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="34.5" customHeight="1" s="15">
       <c r="B25" s="12" t="inlineStr">
@@ -1310,6 +1374,11 @@
           <t>Per-TF K_Threshold_Pct: M5=0.40, M15=0.60, M30=0.60, H1=0.60 (vs preBB v6's single shared K=0.55)</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>THS/THB + THS2/THB2 same engine as BB (6TF, EMA-chase); TP re-pegs via EMA frac</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="34.5" customHeight="1" s="15">
       <c r="B26" s="12" t="inlineStr">
@@ -1357,6 +1426,11 @@
           <t>Per-TF ChaseFraction: M5=0.5, M15=0.5, M30=0.5, H1=0.6</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>NEW: M1 threshold+TP use exact self-consistent band point (Band(P)=P, quadratic solve)</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="34.5" customHeight="1" s="15">
       <c r="B27" s="12" t="inlineStr">
@@ -1404,6 +1478,11 @@
           <t>RSI(14) confirmation gate (InpUseRSIGate=true): SELL only if RSI(shift1)&gt;=50+X, BUY only if RSI&lt;=50-X, X per TF: M5=0(off), M15=10, M30=5, H1=5. Found the losing zone is mid-momentum RSI 50-70, not extreme overbought/oversold.</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>M1_TPBlendFrac=0.75 (TP blended 75% toward the solved point); all other TFs =0 (untouched original)</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="34.5" customHeight="1" s="15">
       <c r="B28" s="12" t="inlineStr">
@@ -1445,6 +1524,11 @@
       <c r="J28" t="inlineStr">
         <is>
           <t>Same TP-chase mechanism as preBB v6 (EMA fraction toward close each bar), InpMaxBarsHold=0</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>LotSize 0.02, Slippage 500, M1 cooldown 0 (was 1), M1 max concurrent 4 (was 3), DailyProfitStopPct 100%</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1760,11 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr"/>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>BB M1-blend: 70/30 split + bootstrap showed the M1 edge is regime-dependent, not stable (train window favored the original snapshot logic, test window favored the blend) - kept on the reasoning that H2-2025 XAUUSD price roughly doubled vs the training period, changing the fixed-price-unit threshold's relative bite. Re-validate if price regime shifts again.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">

</xml_diff>